<commit_message>
Combined AM Calendar for both systems; level the pneumatic periodic months
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vifuQNcyNXj8yaGsTha9n
</commit_message>
<xml_diff>
--- a/training/hydraulic-series/am/AM_Standard_Pneumatic_System.xlsx
+++ b/training/hydraulic-series/am/AM_Standard_Pneumatic_System.xlsx
@@ -1561,7 +1561,7 @@
     <t xml:space="preserve">AM Calendar — ระบบลม · ปี ……</t>
   </si>
   <si>
-    <t xml:space="preserve">D = ทุกวัน · W = รายสัปดาห์ · Q = ทุก 3 เดือน (มี.ค. มิ.ย. ก.ย. ธ.ค. *) · S = ทุก 6 เดือน (มิ.ย. ธ.ค. *) · A = ทุก 1 ปี (ธ.ค. *) · เดือนที่ตรวจตามรอบเป็นข้อเสนอ ให้วางตามแผนหยุดเครื่อง</t>
+    <t xml:space="preserve">D = ทุกวัน · W = รายสัปดาห์ · Q = ทุก 3 เดือน (ม.ค. เม.ย. ก.ค. ต.ค. *) · S = ทุก 6 เดือน (มิ.ย. ธ.ค. *) · A = ทุก 1 ปี (ก.ค. *) · เดือนตามรอบเป็นข้อเสนอ เกลี่ยกับอีกระบบแล้ว (AM_Calendar_Combined.xlsx) ให้วางตามแผนหยุดเครื่อง</t>
   </si>
   <si>
     <t xml:space="preserve">กิจกรรม (CILT)</t>
@@ -6570,26 +6570,26 @@
         <f aca="false">AM_Standard!J7</f>
         <v>HIGH</v>
       </c>
-      <c r="F7" s="16"/>
+      <c r="F7" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G7" s="16"/>
-      <c r="H7" s="28" t="s">
+      <c r="H7" s="16"/>
+      <c r="I7" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I7" s="16"/>
       <c r="J7" s="16"/>
-      <c r="K7" s="28" t="s">
+      <c r="K7" s="16"/>
+      <c r="L7" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L7" s="16"/>
       <c r="M7" s="16"/>
-      <c r="N7" s="28" t="s">
+      <c r="N7" s="16"/>
+      <c r="O7" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O7" s="16"/>
       <c r="P7" s="16"/>
-      <c r="Q7" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q7" s="16"/>
       <c r="R7" s="21" t="s">
         <v>296</v>
       </c>
@@ -7146,26 +7146,26 @@
         <f aca="false">AM_Standard!J18</f>
         <v>CRITICAL</v>
       </c>
-      <c r="F18" s="16"/>
+      <c r="F18" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G18" s="16"/>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I18" s="16"/>
       <c r="J18" s="16"/>
-      <c r="K18" s="28" t="s">
+      <c r="K18" s="16"/>
+      <c r="L18" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L18" s="16"/>
       <c r="M18" s="16"/>
-      <c r="N18" s="28" t="s">
+      <c r="N18" s="16"/>
+      <c r="O18" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O18" s="16"/>
       <c r="P18" s="16"/>
-      <c r="Q18" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q18" s="16"/>
       <c r="R18" s="16" t="s">
         <v>286</v>
       </c>
@@ -7187,26 +7187,26 @@
         <f aca="false">AM_Standard!J19</f>
         <v>CRITICAL</v>
       </c>
-      <c r="F19" s="16"/>
+      <c r="F19" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G19" s="16"/>
-      <c r="H19" s="28" t="s">
+      <c r="H19" s="16"/>
+      <c r="I19" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I19" s="16"/>
       <c r="J19" s="16"/>
-      <c r="K19" s="28" t="s">
+      <c r="K19" s="16"/>
+      <c r="L19" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L19" s="16"/>
       <c r="M19" s="16"/>
-      <c r="N19" s="28" t="s">
+      <c r="N19" s="16"/>
+      <c r="O19" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O19" s="16"/>
       <c r="P19" s="16"/>
-      <c r="Q19" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q19" s="16"/>
       <c r="R19" s="21" t="s">
         <v>383</v>
       </c>
@@ -7228,26 +7228,26 @@
         <f aca="false">AM_Standard!J20</f>
         <v>HIGH</v>
       </c>
-      <c r="F20" s="16"/>
+      <c r="F20" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G20" s="16"/>
-      <c r="H20" s="28" t="s">
+      <c r="H20" s="16"/>
+      <c r="I20" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I20" s="16"/>
       <c r="J20" s="16"/>
-      <c r="K20" s="28" t="s">
+      <c r="K20" s="16"/>
+      <c r="L20" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L20" s="16"/>
       <c r="M20" s="16"/>
-      <c r="N20" s="28" t="s">
+      <c r="N20" s="16"/>
+      <c r="O20" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O20" s="16"/>
       <c r="P20" s="16"/>
-      <c r="Q20" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q20" s="16"/>
       <c r="R20" s="16" t="s">
         <v>286</v>
       </c>
@@ -7275,14 +7275,14 @@
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
       <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
+      <c r="L21" s="33" t="s">
+        <v>471</v>
+      </c>
       <c r="M21" s="16"/>
       <c r="N21" s="16"/>
       <c r="O21" s="16"/>
       <c r="P21" s="16"/>
-      <c r="Q21" s="33" t="s">
-        <v>471</v>
-      </c>
+      <c r="Q21" s="16"/>
       <c r="R21" s="21" t="s">
         <v>398</v>
       </c>
@@ -7383,26 +7383,26 @@
         <f aca="false">AM_Standard!J24</f>
         <v>HIGH</v>
       </c>
-      <c r="F24" s="16"/>
+      <c r="F24" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G24" s="16"/>
-      <c r="H24" s="28" t="s">
+      <c r="H24" s="16"/>
+      <c r="I24" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I24" s="16"/>
       <c r="J24" s="16"/>
-      <c r="K24" s="28" t="s">
+      <c r="K24" s="16"/>
+      <c r="L24" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L24" s="16"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="28" t="s">
+      <c r="N24" s="16"/>
+      <c r="O24" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O24" s="16"/>
       <c r="P24" s="16"/>
-      <c r="Q24" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q24" s="16"/>
       <c r="R24" s="16" t="s">
         <v>286</v>
       </c>
@@ -7424,26 +7424,26 @@
         <f aca="false">AM_Standard!J25</f>
         <v>LOW</v>
       </c>
-      <c r="F25" s="16"/>
+      <c r="F25" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G25" s="16"/>
-      <c r="H25" s="28" t="s">
+      <c r="H25" s="16"/>
+      <c r="I25" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I25" s="16"/>
       <c r="J25" s="16"/>
-      <c r="K25" s="28" t="s">
+      <c r="K25" s="16"/>
+      <c r="L25" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L25" s="16"/>
       <c r="M25" s="16"/>
-      <c r="N25" s="28" t="s">
+      <c r="N25" s="16"/>
+      <c r="O25" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O25" s="16"/>
       <c r="P25" s="16"/>
-      <c r="Q25" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q25" s="16"/>
       <c r="R25" s="21" t="s">
         <v>383</v>
       </c>
@@ -7471,14 +7471,14 @@
       <c r="I26" s="16"/>
       <c r="J26" s="16"/>
       <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
+      <c r="L26" s="33" t="s">
+        <v>471</v>
+      </c>
       <c r="M26" s="16"/>
       <c r="N26" s="16"/>
       <c r="O26" s="16"/>
       <c r="P26" s="16"/>
-      <c r="Q26" s="33" t="s">
-        <v>471</v>
-      </c>
+      <c r="Q26" s="16"/>
       <c r="R26" s="21" t="s">
         <v>398</v>
       </c>
@@ -7506,14 +7506,14 @@
       <c r="I27" s="16"/>
       <c r="J27" s="16"/>
       <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
+      <c r="L27" s="33" t="s">
+        <v>471</v>
+      </c>
       <c r="M27" s="16"/>
       <c r="N27" s="16"/>
       <c r="O27" s="16"/>
       <c r="P27" s="16"/>
-      <c r="Q27" s="33" t="s">
-        <v>471</v>
-      </c>
+      <c r="Q27" s="16"/>
       <c r="R27" s="21" t="s">
         <v>398</v>
       </c>
@@ -7557,26 +7557,26 @@
         <f aca="false">AM_Standard!J29</f>
         <v>HIGH</v>
       </c>
-      <c r="F29" s="16"/>
+      <c r="F29" s="28" t="s">
+        <v>469</v>
+      </c>
       <c r="G29" s="16"/>
-      <c r="H29" s="28" t="s">
+      <c r="H29" s="16"/>
+      <c r="I29" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="I29" s="16"/>
       <c r="J29" s="16"/>
-      <c r="K29" s="28" t="s">
+      <c r="K29" s="16"/>
+      <c r="L29" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="L29" s="16"/>
       <c r="M29" s="16"/>
-      <c r="N29" s="28" t="s">
+      <c r="N29" s="16"/>
+      <c r="O29" s="28" t="s">
         <v>469</v>
       </c>
-      <c r="O29" s="16"/>
       <c r="P29" s="16"/>
-      <c r="Q29" s="28" t="s">
-        <v>469</v>
-      </c>
+      <c r="Q29" s="16"/>
       <c r="R29" s="16" t="s">
         <v>286</v>
       </c>
@@ -7604,14 +7604,14 @@
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
       <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
+      <c r="L30" s="33" t="s">
+        <v>471</v>
+      </c>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
       <c r="O30" s="16"/>
       <c r="P30" s="16"/>
-      <c r="Q30" s="33" t="s">
-        <v>471</v>
-      </c>
+      <c r="Q30" s="16"/>
       <c r="R30" s="21" t="s">
         <v>398</v>
       </c>

</xml_diff>